<commit_message>
first commit for v2
</commit_message>
<xml_diff>
--- a/MIR/bin/Debug/net8.0-windows/data.xlsx
+++ b/MIR/bin/Debug/net8.0-windows/data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Id</t>
   </si>
@@ -39,13 +39,13 @@
     <t>CreatedAt</t>
   </si>
   <si>
-    <t>a4aa2c84-6c45-49af-9aee-943ba8fb1535</t>
+    <t>f4f3f874-b984-498b-99bb-4417371526a9</t>
   </si>
   <si>
     <t>admin</t>
   </si>
   <si>
-    <t>$2a$11$GsKxbnIankQkmNnu8zD4xuYvpD86TRz3UM3MLKaOujv9L8i4Qu9Q.</t>
+    <t>$2a$11$VOP4cmv9IqpGbDD1Y8X9NO39xTkZ.I.y4tQRpCxtkcZUpd9hyMcBC</t>
   </si>
   <si>
     <t>Administrator</t>
@@ -54,7 +54,7 @@
     <t>Admin</t>
   </si>
   <si>
-    <t>2026-02-01T20:06:13.5441986+08:00</t>
+    <t>2026-02-01T19:54:53.6861593+08:00</t>
   </si>
   <si>
     <t>Code</t>
@@ -84,6 +84,60 @@
     <t>LastUpdated</t>
   </si>
   <si>
+    <t>aaab711a-4390-489e-beaa-f56543e57280</t>
+  </si>
+  <si>
+    <t>MAT-202602012013</t>
+  </si>
+  <si>
+    <t>egg</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>pcs</t>
+  </si>
+  <si>
+    <t>Raw Materials</t>
+  </si>
+  <si>
+    <t>2026-02-01T20:13:07.2262291+08:00</t>
+  </si>
+  <si>
+    <t>d92829e8-7789-43f8-a1dd-8565fe9cca59</t>
+  </si>
+  <si>
+    <t>rice</t>
+  </si>
+  <si>
+    <t>2026-02-01T20:13:19.7691453+08:00</t>
+  </si>
+  <si>
+    <t>5d171112-732a-45cd-a90b-3325e392ef33</t>
+  </si>
+  <si>
+    <t>sambal</t>
+  </si>
+  <si>
+    <t>2026-02-01T20:13:30.2899484+08:00</t>
+  </si>
+  <si>
+    <t>16762699-04e6-46ed-af6f-7552f9279a3f</t>
+  </si>
+  <si>
+    <t>PRD-202602012013</t>
+  </si>
+  <si>
+    <t>nasi lemak</t>
+  </si>
+  <si>
+    <t>Finished Goods</t>
+  </si>
+  <si>
+    <t>2026-02-01T20:13:44.4094990+08:00</t>
+  </si>
+  <si>
     <t>ProductId</t>
   </si>
   <si>
@@ -91,6 +145,15 @@
   </si>
   <si>
     <t>Quantity</t>
+  </si>
+  <si>
+    <t>62d17645-657c-48bd-a267-81dff1f6038b</t>
+  </si>
+  <si>
+    <t>f3e36b80-ea1e-4903-a797-ea847348d19a</t>
+  </si>
+  <si>
+    <t>15eeb5b3-cfc0-40f8-ab6f-b9d179cc9a46</t>
   </si>
   <si>
     <t>Type</t>
@@ -204,7 +267,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -239,6 +302,102 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="0">
+        <v>50</v>
+      </c>
+      <c r="G2" s="0">
+        <v>20</v>
+      </c>
+      <c r="H2" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="0">
+        <v>100</v>
+      </c>
+      <c r="G3" s="0">
+        <v>20</v>
+      </c>
+      <c r="H3" s="0">
+        <v>1</v>
+      </c>
+      <c r="I3" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="0">
+        <v>50</v>
+      </c>
+      <c r="G4" s="0">
+        <v>10</v>
+      </c>
+      <c r="H4" s="0">
+        <v>0.6</v>
+      </c>
+      <c r="I4" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="0" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>
@@ -246,7 +405,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -272,6 +431,29 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <headerFooter/>
 </worksheet>
@@ -279,7 +461,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -287,13 +469,55 @@
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1" s="0" t="s">
-        <v>24</v>
+      <c r="D2" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="0">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -311,22 +535,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>